<commit_message>
Esiti test direttivo (Giulia): riepilogo pagamenti snello, ospite, sfide, chip saldo
- Riepilogo pagamenti: in evidenza "Paghi tu / Hai pagato" con quanto esce davvero
  dal saldo, scomposizione solo se serve (tua quota, ospiti, quote coperte); soci
  con credito su una riga compatta. Corretto il caso "Prenota per Socio" in cui il
  prenotante non gioca (prima vedeva "Tua quota"). Tolti "Saldo dopo l'operazione"
  e "Totale prenotazione".
- Aggiunta ospite: bottoni "Aggiungi" / "Annulla" al posto della sola spunta.
- Cerco Partita: le sfide accettate spariscono da "Le mie sfide".
- Chip saldo accanto all'avatar (UserNav) su tutte le pagine; tile dashboard invariato.
- Storico movimenti: campo e giorno della partita, data del movimento distinta.
- Excel del test compilato da Giulia; test e2e aggiornati ai nuovi testi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test-Portafoglio-Direttivo.xlsx
+++ b/docs/Test-Portafoglio-Direttivo.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC32935F-0B31-4822-90DD-4C0728A4E0B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Leggimi" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Prove" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Impressioni" state="visible" r:id="rId6"/>
+    <sheet name="Leggimi" sheetId="1" r:id="rId1"/>
+    <sheet name="Prove" sheetId="2" r:id="rId2"/>
+    <sheet name="Impressioni" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Prove'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">Prove!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="124">
   <si>
     <t>Prova del Portafoglio — Canepacce</t>
   </si>
@@ -90,15 +94,9 @@
     <t>Mario Prova</t>
   </si>
   <si>
-    <t>socio.prova1@canepacce.test · password: ______________ · parte con credito</t>
-  </si>
-  <si>
     <t>Luigi Prova</t>
   </si>
   <si>
-    <t>socio.prova2@canepacce.test · password: ______________ · parte senza credito</t>
-  </si>
-  <si>
     <t>Carta di prova</t>
   </si>
   <si>
@@ -132,9 +130,6 @@
     <t>Segui l'ordine. Celle gialle = da compilare.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nome: </t>
-  </si>
-  <si>
     <t>N.</t>
   </si>
   <si>
@@ -150,11 +145,11 @@
     <t>Cosa dovresti vedere</t>
   </si>
   <si>
-    <t xml:space="preserve">Ci sei
+    <t>Ci sei
 riuscito?</t>
   </si>
   <si>
-    <t xml:space="preserve">Era
+    <t>Era
 chiaro?</t>
   </si>
   <si>
@@ -170,7 +165,7 @@
     <t>Mario</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Entra con l'account di Mario.
+    <t>1. Entra con l'account di Mario.
 2. Nella pagina principale cerca il riquadro "Il mio Portafoglio" e premi "Vai al Portafoglio".</t>
   </si>
   <si>
@@ -183,13 +178,13 @@
     <t>Giocare con chi non ha credito</t>
   </si>
   <si>
-    <t xml:space="preserve">1. "Prenota un Campo" → scegli un giorno della SETTIMANA PROSSIMA, un campo, un orario di giorno (es. 10:00) e "Singolare".
+    <t>1. "Prenota un Campo" → scegli un giorno della SETTIMANA PROSSIMA, un campo, un orario di giorno (es. 10:00) e "Singolare".
 2. Nei partecipanti cerca e aggiungi "Luigi Prova" (che non ha credito).
 3. Premi "Conferma Prenotazione" e LEGGI con calma il riepilogo.
 4. Conferma.</t>
   </si>
   <si>
-    <t xml:space="preserve">Un riquadro arancione avvisa che Luigi non ha credito e che la sua quota la paghi tu. Il bottone dice quanto paghi in tutto. Dopo la conferma il riepilogo finale lo ripete.
+    <t>Un riquadro arancione avvisa che Luigi non ha credito e che la sua quota la paghi tu. Il bottone dice quanto paghi in tutto. Dopo la conferma il riepilogo finale lo ripete.
 Domanda: prima di pagare avevi capito esattamente quanto ti sarebbe costato e perché?</t>
   </si>
   <si>
@@ -199,19 +194,19 @@
     <t>Luigi</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Esci ed entra come Luigi (saldo €0).
+    <t>1. Esci ed entra come Luigi (saldo €0).
 2. Prova a prenotare un Singolare con "Mario Prova" (settimana prossima, un altro orario).
 3. Leggi il riquadro rosso, poi premi il bottone verde "Ricarica €…".</t>
   </si>
   <si>
-    <t xml:space="preserve">Il riquadro rosso spiega quanto serve, quanto hai e quanto ti manca. Il bottone ti porta al portafoglio con l'importo già scritto.
+    <t>Il riquadro rosso spiega quanto serve, quanto hai e quanto ti manca. Il bottone ti porta al portafoglio con l'importo già scritto.
 Domanda: avresti saputo cosa fare anche senza questa guida?</t>
   </si>
   <si>
     <t>Ricaricare con la carta</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Nella pagina del portafoglio cambia l'importo in 10 e premi "Ricarica".
+    <t>1. Nella pagina del portafoglio cambia l'importo in 10 e premi "Ricarica".
 2. Nella pagina di pagamento usa la carta di prova 4242 4242 4242 4242, scadenza 12/30, CVC 123.
 3. Paga e aspetta di tornare nell'app.</t>
   </si>
@@ -222,7 +217,7 @@
     <t>Ognuno paga la sua quota</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Premi "Torna a prenotare" e rifai la prenotazione della prova 3.
+    <t>1. Premi "Torna a prenotare" e rifai la prenotazione della prova 3.
 2. Leggi il riepilogo e conferma.</t>
   </si>
   <si>
@@ -232,7 +227,7 @@
     <t>Cambiare idea sul pagamento</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Nel portafoglio premi "€10".
+    <t>1. Nel portafoglio premi "€10".
 2. Nella pagina di pagamento NON pagare: torna indietro.</t>
   </si>
   <si>
@@ -242,12 +237,12 @@
     <t>Doppio con un ospite</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Entra come Mario.
+    <t>1. Entra come Mario.
 2. Prenota un "Doppio" di 1 ora (settimana prossima) con: Luigi, un ospite (premi "Ospite" e scrivi un nome) e "Da definire".
 3. Leggi il riepilogo e conferma.</t>
   </si>
   <si>
-    <t xml:space="preserve">La tua quota è più alta perché comprende l'ospite e il "Da definire" (c'è scritto). Luigi paga solo la sua.
+    <t>La tua quota è più alta perché comprende l'ospite e il "Da definire" (c'è scritto). Luigi paga solo la sua.
 Domanda: si capisce perché paghi più di Luigi?</t>
   </si>
   <si>
@@ -257,7 +252,7 @@
     <t>Allungare una prenotazione</t>
   </si>
   <si>
-    <t xml:space="preserve">1. "I miei Campi" → sul Doppio della prova 7 premi "Modifica".
+    <t>1. "I miei Campi" → sul Doppio della prova 7 premi "Modifica".
 2. Aggiungi l'ora successiva e premi "Salva Modifiche".</t>
   </si>
   <si>
@@ -267,18 +262,18 @@
     <t>Accorciare una prenotazione</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Sulla stessa prenotazione (ora di 2 ore) premi "Modifica".
+    <t>1. Sulla stessa prenotazione (ora di 2 ore) premi "Modifica".
 2. Togli un'ora e premi "Salva Modifiche".</t>
   </si>
   <si>
-    <t xml:space="preserve">In alto: "Con questa modifica non paghi nulla: ricevi un rimborso". Le righe "Rimborsi" hanno il "+" davanti. Il bottone dice "Conferma e ricevi €…".
+    <t>In alto: "Con questa modifica non paghi nulla: ricevi un rimborso". Le righe "Rimborsi" hanno il "+" davanti. Il bottone dice "Conferma e ricevi €…".
 Domanda IMPORTANTE: c'è qualcosa che ti fa pensare di pagare di nuovo?</t>
   </si>
   <si>
     <t>Annullare una prenotazione</t>
   </si>
   <si>
-    <t xml:space="preserve">1. In "I miei Campi" premi il cestino rosso sul Doppio.
+    <t>1. In "I miei Campi" premi il cestino rosso sul Doppio.
 2. Leggi la finestra, poi premi "Elimina".</t>
   </si>
   <si>
@@ -291,11 +286,11 @@
     <t>Mario e Luigi</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Apri "Il mio Portafoglio" di Mario e leggi tutti i movimenti.
+    <t>1. Apri "Il mio Portafoglio" di Mario e leggi tutti i movimenti.
 2. Fai lo stesso con Luigi.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ogni riga dice cos'è (ricarica, prenotazione, quota coperta per un altro socio, rimborso) con data e importo, e il saldo torna.
+    <t>Ogni riga dice cos'è (ricarica, prenotazione, quota coperta per un altro socio, rimborso) con data e importo, e il saldo torna.
 Domanda: c'è una riga che non sapresti spiegare a un altro socio?</t>
   </si>
   <si>
@@ -308,7 +303,7 @@
     <t>Luigi, poi Mario</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Come Luigi: "Cerco Partita" → pubblica una sfida Singolare per un giorno della settimana DOPO la prossima (l'app non va oltre 14 giorni da oggi).
+    <t>1. Come Luigi: "Cerco Partita" → pubblica una sfida Singolare per un giorno della settimana DOPO la prossima (l'app non va oltre 14 giorni da oggi).
 2. Come Mario: "Cerco Partita" → accetta la sfida di Luigi → nella pagina "Conferma Sfida" premi "Accetta e Prenota" e leggi il riepilogo.</t>
   </si>
   <si>
@@ -318,7 +313,7 @@
     <t>Prenotare per un altro socio</t>
   </si>
   <si>
-    <t xml:space="preserve">1. "Prenota per Socio" → un giorno della settimana DOPO la prossima (entro 14 giorni), campo, orario, "Singolare".
+    <t>1. "Prenota per Socio" → un giorno della settimana DOPO la prossima (entro 14 giorni), campo, orario, "Singolare".
 2. Aggiungi Luigi e un ospite. Conferma.</t>
   </si>
   <si>
@@ -334,7 +329,7 @@
     <t>Admin</t>
   </si>
   <si>
-    <t xml:space="preserve">1. "Pannello Admin" → "Portafogli Soci" → cerca Luigi.
+    <t>1. "Pannello Admin" → "Portafogli Soci" → cerca Luigi.
 2. "Accredita Contanti": €5 con una nota.</t>
   </si>
   <si>
@@ -344,7 +339,7 @@
     <t>Prenotare per chi paga in contanti</t>
   </si>
   <si>
-    <t xml:space="preserve">1. "Pannello Admin" → "Prenotazioni" → clicca uno slot libero, scrivi nome e cognome, "Crea".
+    <t>1. "Pannello Admin" → "Prenotazioni" → clicca uno slot libero, scrivi nome e cognome, "Crea".
 2. Clicca l'icona "€" sullo slot.</t>
   </si>
   <si>
@@ -382,64 +377,135 @@
   </si>
   <si>
     <t>6. Altro che vuoi segnalare:</t>
+  </si>
+  <si>
+    <t>socio.prova1@canepacce.test · password: ____prova1______ · parte con credito</t>
+  </si>
+  <si>
+    <t>socio.prova2@canepacce.test · password: ____prova2______ · parte senza credito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tile : Portafoglio , Sezione : Elenco movimenti , affianco al testo prenotazione campo specificare meglio anche quale campo e quale giorno mentre nel testo sottostante che dice in che momento è stata effettuata la prenotazione magari è meglio specificarlo che è un data diversa </t>
+  </si>
+  <si>
+    <t>Sì</t>
+  </si>
+  <si>
+    <t>Chiarissimo</t>
+  </si>
+  <si>
+    <t>Abbastanza</t>
+  </si>
+  <si>
+    <t>Poco</t>
+  </si>
+  <si>
+    <t>il tile "il mio portafoglio" al momento è sconnesso a livello concettuale con gli altri già presenti, gli va trovata una collocazione diversa, forse accanto all'icona del profilo? Boh indaga.</t>
+  </si>
+  <si>
+    <t>nel caso in cui si sta pagando la quota anche per un socio che non ha credito, per come sono gestite le etichette ora , sembra che io stia pagando solo la mia quota perché è più in risalto di quanto in realtà pagherò dopo aver effettuato la prenotazione , in questo caso è fuorviante l'info tra parentesi , dobbiamo risolvere questa ambiguità.</t>
+  </si>
+  <si>
+    <t>1) se il socio aggiunto alla partita ha credito ed è quindi in grado di pagarsi il campo da solo , il riepilogo deve essere più snello , per la quota pagata dall'altro socio basta una sola etichetta che dice che ha il saldo e paga la sua parte, così mettiamo più enfasi alla quota effettiva pagata da chi sta facendo la prenotazione.
+2) la funzionalità di aggiunta ospite è al momento poco parlante, non si capisce che la spunta affianco va cliccata per salvare l'ospite</t>
+  </si>
+  <si>
+    <t>la sfida una volta accettata deve eliminarsi dalla visualizzazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sono stati scalati dei soldi anche nel caso di una prenotazione non andata a buon fine , facciamo attenzione! </t>
+  </si>
+  <si>
+    <t>Per niente</t>
+  </si>
+  <si>
+    <t>Nome:  Giulia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF2E6B3D"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF6B7280"/>
+      <sz val="13"/>
+      <color rgb="FFD96B27"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF2E6B3D"/>
-      <sz val="13"/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFD96B27"/>
-      <sz val="13"/>
+      <sz val="12"/>
+      <color rgb="FF2E6B3D"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="18"/>
+      <sz val="11"/>
+      <color rgb="FF2E6B3D"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+      <color rgb="FFD96B27"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF2E6B3D"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF2E6B3D"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFD96B27"/>
-      <sz val="12"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -512,11 +578,54 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -524,76 +633,28 @@
       <alignment indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF15803D"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -619,22 +680,22 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF15803D"/>
+        <color rgb="FF4D7C0F"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFDCFCE7"/>
+          <fgColor rgb="FFECFCCB"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <color rgb="FF4D7C0F"/>
+        <color rgb="FF15803D"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFECFCCB"/>
+          <fgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -657,6 +718,17 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF15803D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -994,194 +1066,201 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="92" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+    </row>
+    <row r="2" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+    </row>
+    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="C4" s="17"/>
+    </row>
+    <row r="5" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="6" t="s">
+    <row r="6" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="3"/>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
+      <c r="C8" s="17"/>
+    </row>
+    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
+    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="4" t="s">
+    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
+    <row r="12" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
+    <row r="13" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
+    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="8" t="s">
+    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="8"/>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
+      <c r="C16" s="18"/>
+    </row>
+    <row r="17" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="4" t="s">
+    <row r="18" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="24" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="24" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="9" t="s">
+    <row r="21" spans="2:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C21" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="4" t="s">
+    <row r="23" spans="2:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C23" s="18"/>
+    </row>
+    <row r="24" spans="2:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="8" t="s">
+      <c r="C24" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="8"/>
-    </row>
-    <row r="24" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24" s="4" t="s">
+    </row>
+    <row r="25" spans="2:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C25" s="2" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="25" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B23:C23"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C18" r:id="rId1" xr:uid="{B68D40A5-FE84-44B1-8F3E-94FDFB5A2086}"/>
+    <hyperlink ref="C19" r:id="rId2" xr:uid="{4446031C-E771-4A71-80E9-42C6901ECE4A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Informazione ad uso interno - Internal use information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -1192,576 +1271,613 @@
     <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+    </row>
+    <row r="4" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="B4" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13" t="s">
+      <c r="C4" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-    </row>
-    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="D4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="E4" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="F4" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="G4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="H4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="14" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+    </row>
+    <row r="6" spans="1:8" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>1</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="C6" s="10" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="D6" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-    </row>
-    <row r="6" ht="55" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
-        <v>1</v>
-      </c>
-      <c r="B6" s="17" t="s">
+      <c r="E6" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="F6" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+    </row>
+    <row r="8" spans="1:8" ht="129.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>2</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="C8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="E8" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-    </row>
-    <row r="8" ht="130" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="16">
-        <v>2</v>
-      </c>
-      <c r="B8" s="17" t="s">
+      <c r="F8" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>3</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="C9" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="D9" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="21"/>
-    </row>
-    <row r="9" ht="85" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
-        <v>3</v>
-      </c>
-      <c r="B9" s="17" t="s">
+      <c r="E9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="F9" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H9" s="13"/>
+    </row>
+    <row r="10" spans="1:8" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>4</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="C10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E10" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="21"/>
-    </row>
-    <row r="10" ht="85" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="16">
-        <v>4</v>
-      </c>
-      <c r="B10" s="17" t="s">
+      <c r="F10" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H10" s="13"/>
+    </row>
+    <row r="11" spans="1:8" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>5</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="19" t="s">
+      <c r="C11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E11" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="21"/>
-    </row>
-    <row r="11" ht="85" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="16">
-        <v>5</v>
-      </c>
-      <c r="B11" s="17" t="s">
+      <c r="F11" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H11" s="13"/>
+    </row>
+    <row r="12" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>6</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="19" t="s">
+      <c r="C12" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E12" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="21"/>
-    </row>
-    <row r="12" ht="55" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="16">
-        <v>6</v>
-      </c>
-      <c r="B12" s="17" t="s">
+      <c r="F12" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H12" s="13"/>
+    </row>
+    <row r="13" spans="1:8" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>7</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="19" t="s">
+      <c r="C13" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E13" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="21"/>
-    </row>
-    <row r="13" ht="85" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="16">
-        <v>7</v>
-      </c>
-      <c r="B13" s="17" t="s">
+      <c r="F13" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="19" t="s">
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+    </row>
+    <row r="15" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>8</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="C15" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="21"/>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+      <c r="E15" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-    </row>
-    <row r="15" ht="55" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
-        <v>8</v>
-      </c>
-      <c r="B15" s="17" t="s">
+      <c r="F15" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H15" s="13"/>
+    </row>
+    <row r="16" spans="1:8" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <v>9</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C15" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="19" t="s">
+      <c r="C16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E16" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="21"/>
-    </row>
-    <row r="16" ht="85" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="16">
-        <v>9</v>
-      </c>
-      <c r="B16" s="17" t="s">
+      <c r="F16" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H16" s="13"/>
+    </row>
+    <row r="17" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
+        <v>10</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D16" s="19" t="s">
+      <c r="C17" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E17" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="21"/>
-    </row>
-    <row r="17" ht="70" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="16">
-        <v>10</v>
-      </c>
-      <c r="B17" s="17" t="s">
+      <c r="F17" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H17" s="13"/>
+    </row>
+    <row r="18" spans="1:8" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="8">
+        <v>11</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" s="19" t="s">
+      <c r="C18" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="D18" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="21"/>
-    </row>
-    <row r="18" ht="85" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="16">
-        <v>11</v>
-      </c>
-      <c r="B18" s="17" t="s">
+      <c r="E18" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="F18" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H18" s="13"/>
+    </row>
+    <row r="19" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+    </row>
+    <row r="20" spans="1:8" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="8">
+        <v>12</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="C20" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="21"/>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="D20" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-    </row>
-    <row r="20" ht="100" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="16">
-        <v>12</v>
-      </c>
-      <c r="B20" s="17" t="s">
+      <c r="E20" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="F20" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="8">
+        <v>13</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="C21" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E21" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="21"/>
-    </row>
-    <row r="21" ht="70" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="16">
-        <v>13</v>
-      </c>
-      <c r="B21" s="17" t="s">
+      <c r="F21" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="19" t="s">
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+    </row>
+    <row r="23" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
+        <v>14</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="C23" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="21"/>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="D23" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-    </row>
-    <row r="23" ht="55" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
-        <v>14</v>
-      </c>
-      <c r="B23" s="17" t="s">
+      <c r="E23" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="13"/>
+    </row>
+    <row r="24" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
+        <v>15</v>
+      </c>
+      <c r="B24" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="C24" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E24" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="21"/>
-    </row>
-    <row r="24" ht="55" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="16">
-        <v>15</v>
-      </c>
-      <c r="B24" s="17" t="s">
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="13"/>
+    </row>
+    <row r="25" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="8">
+        <v>16</v>
+      </c>
+      <c r="B25" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D24" s="19" t="s">
+      <c r="C25" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E25" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="21"/>
-    </row>
-    <row r="25" ht="55" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="16">
-        <v>16</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="E25" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="21"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F25">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"Sì"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"In parte"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G25">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"Chiarissimo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
       <formula>"Abbastanza"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
       <formula>"Poco"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
       <formula>"Per niente"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F10:F13">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F8:F13 F6 F23:F25 F20:F21 F15:F18" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Sì,No,In parte,Non provato"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F15:F18">
-      <formula1>"Sì,No,In parte,Non provato"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F20:F21">
-      <formula1>"Sì,No,In parte,Non provato"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F23:F25">
-      <formula1>"Sì,No,In parte,Non provato"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F6">
-      <formula1>"Sì,No,In parte,Non provato"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Sì, No, In parte, Non provato" sqref="F8:F13">
-      <formula1>"Sì,No,In parte,Non provato"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G10:G13">
-      <formula1>"Chiarissimo,Abbastanza,Poco,Per niente"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G15:G18">
-      <formula1>"Chiarissimo,Abbastanza,Poco,Per niente"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G20:G21">
-      <formula1>"Chiarissimo,Abbastanza,Poco,Per niente"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G23:G25">
-      <formula1>"Chiarissimo,Abbastanza,Poco,Per niente"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G6">
-      <formula1>"Chiarissimo,Abbastanza,Poco,Per niente"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G8:G13">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Scegli dal menu: Chiarissimo, Abbastanza, Poco, Per niente" sqref="G8:G13 G6 G23:G25 G20:G21 G15:G18" xr:uid="{00000000-0002-0000-0100-000006000000}">
       <formula1>"Chiarissimo,Abbastanza,Poco,Per niente"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Informazione ad uso interno - Internal use information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+    </row>
+    <row r="4" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="14"/>
+    </row>
+    <row r="5" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="C5" s="14"/>
+    </row>
+    <row r="6" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-    </row>
-    <row r="4" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+      <c r="C6" s="14"/>
+    </row>
+    <row r="7" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="23"/>
-    </row>
-    <row r="5" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="C7" s="14"/>
+    </row>
+    <row r="8" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="23"/>
-    </row>
-    <row r="6" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
+      <c r="C8" s="14"/>
+    </row>
+    <row r="9" spans="1:3" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="23"/>
-    </row>
-    <row r="7" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C7" s="23"/>
-    </row>
-    <row r="8" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C8" s="23"/>
-    </row>
-    <row r="9" ht="70" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1769,6 +1885,9 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Informazione ad uso interno - Internal use information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>